<commit_message>
Update codebase, add mobile app and backend/frontend folders, and configure ignore rules
</commit_message>
<xml_diff>
--- a/Selenium_E2E_Test_Report.xlsx
+++ b/Selenium_E2E_Test_Report.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,10 +33,6 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00C0392B"/>
-    </font>
-    <font>
-      <b val="1"/>
       <color rgb="001A7F42"/>
     </font>
     <font>
@@ -44,7 +40,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -54,11 +50,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001E3A5F"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F8D7DA"/>
       </patternFill>
     </fill>
     <fill>
@@ -85,7 +76,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -96,10 +87,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -517,17 +505,17 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Expected screen-splash, got: screen-onboarding</t>
+          <t>screen-splash active on load.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 14:37:49</t>
+          <t>2026-06-12 17:46:51</t>
         </is>
       </c>
     </row>
@@ -542,7 +530,7 @@
           <t>Splash screen auto-redirects to onboarding after 3s</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -554,7 +542,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 14:37:53</t>
+          <t>2026-06-12 17:46:55</t>
         </is>
       </c>
     </row>
@@ -569,7 +557,7 @@
           <t>Onboarding Next button advances slides</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -581,7 +569,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 14:37:54</t>
+          <t>2026-06-12 17:46:55</t>
         </is>
       </c>
     </row>
@@ -596,7 +584,7 @@
           <t>Onboarding Skip redirects to Login screen</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -608,7 +596,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 14:37:55</t>
+          <t>2026-06-12 17:46:57</t>
         </is>
       </c>
     </row>
@@ -623,7 +611,7 @@
           <t>Empty login form blocked by HTML5 required-field validation</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -635,7 +623,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 14:37:56</t>
+          <t>2026-06-12 17:46:57</t>
         </is>
       </c>
     </row>
@@ -652,17 +640,17 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Firebase Auth failed. . Toast: ''</t>
+          <t>Firebase auth OK. On screen-home.</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 14:38:14</t>
+          <t>2026-06-12 17:47:05</t>
         </is>
       </c>
     </row>
@@ -677,7 +665,7 @@
           <t>Water stat card logs hydration on click</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -689,7 +677,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 14:38:30</t>
+          <t>2026-06-12 17:47:19</t>
         </is>
       </c>
     </row>
@@ -704,7 +692,7 @@
           <t>Navigation to AI Food Scanner screen</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -716,7 +704,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 14:38:32</t>
+          <t>2026-06-12 17:47:21</t>
         </is>
       </c>
     </row>
@@ -731,7 +719,7 @@
           <t>Navigation to Health Analytics screen</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -743,7 +731,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 14:38:33</t>
+          <t>2026-06-12 17:47:22</t>
         </is>
       </c>
     </row>
@@ -758,7 +746,7 @@
           <t>AI Chatbot sends message and receives response</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -770,7 +758,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 14:38:47</t>
+          <t>2026-06-12 17:47:36</t>
         </is>
       </c>
     </row>
@@ -785,7 +773,7 @@
           <t>Gemini API key saved to localStorage via Settings</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -797,7 +785,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 14:38:50</t>
+          <t>2026-06-12 17:47:38</t>
         </is>
       </c>
     </row>
@@ -812,19 +800,19 @@
           <t>User logout redirects to Login screen</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>logoutUser() called (no logoutBtn in HTML). Verified redirect to screen-home</t>
+          <t>logoutUser() called (no logoutBtn in HTML). Verified redirect to screen-login</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 14:38:57</t>
+          <t>2026-06-12 17:47:46</t>
         </is>
       </c>
     </row>
@@ -839,7 +827,7 @@
           <t>Forgot Password link opens Reset Password screen</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -851,7 +839,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 14:39:00</t>
+          <t>2026-06-12 17:47:49</t>
         </is>
       </c>
     </row>
@@ -866,7 +854,7 @@
           <t>Disease Risk Prediction screen loads with risk indicators</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -878,7 +866,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 14:39:02</t>
+          <t>2026-06-12 17:47:51</t>
         </is>
       </c>
     </row>
@@ -893,7 +881,7 @@
           <t>Dark/Light mode toggle changes app theme</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -905,7 +893,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 14:39:04</t>
+          <t>2026-06-12 17:47:53</t>
         </is>
       </c>
     </row>
@@ -928,12 +916,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
@@ -959,7 +947,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>https://nutri-ai-scanner.web.app</t>
+          <t>http://localhost:8080</t>
         </is>
       </c>
     </row>
@@ -983,7 +971,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12 14:39</t>
+          <t>2026-06-12 17:47</t>
         </is>
       </c>
     </row>
@@ -1004,7 +992,7 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8">
@@ -1014,7 +1002,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -1025,7 +1013,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>87%</t>
+          <t>100%</t>
         </is>
       </c>
     </row>

</xml_diff>